<commit_message>
ly: correct stale provisional wording in PMC v3
</commit_message>
<xml_diff>
--- a/results/ly/task3_natural_trial/pmc_oa_v2_final_trial_set_v3_2026-10-04.xlsx
+++ b/results/ly/task3_natural_trial/pmc_oa_v2_final_trial_set_v3_2026-10-04.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Rb8aded185a264048"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Rfd5c7def923e4d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Rd2a9a5c0088f4b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Re0da84f8729c48f2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -33,9 +33,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">证据状态</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">已定位 / 待定位 / 源文缺失 / 不适用；证据状态不是准确性标签。</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">定位口径</x:t>
@@ -1292,8 +1289,8 @@
       <x:c r="A8" s="11" t="s">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B8" s="12" t="s">
-        <x:v>8</x:v>
+      <x:c r="B8" s="12" t="str">
+        <x:v>本批 20 条均为已定位；证据状态不是准确性标签。</x:v>
       </x:c>
       <x:c r="C8" s="10"/>
       <x:c r="D8" s="10"/>
@@ -1304,10 +1301,10 @@
     </x:row>
     <x:row r="9" ht="15" customHeight="1">
       <x:c r="A9" s="11" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="12" t="s">
         <x:v>9</x:v>
-      </x:c>
-      <x:c r="B9" s="12" t="s">
-        <x:v>10</x:v>
       </x:c>
       <x:c r="C9" s="10"/>
       <x:c r="D9" s="10"/>
@@ -1318,7 +1315,7 @@
     </x:row>
     <x:row r="10" ht="15" customHeight="1">
       <x:c r="A10" s="11" t="s">
-        <x:v>11</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B10" s="12" t="str">
         <x:v>双方原始标签保留；分歧写入 adjudication_reason，NOT-ACCURATE 只在比较统计时规范化为 NOT_ACCURATE。</x:v>
@@ -1342,10 +1339,10 @@
     </x:row>
     <x:row r="12" ht="15" customHeight="1">
       <x:c r="A12" s="13" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B12" s="12" t="s">
         <x:v>12</x:v>
-      </x:c>
-      <x:c r="B12" s="12" t="s">
-        <x:v>13</x:v>
       </x:c>
       <x:c r="C12" s="10"/>
       <x:c r="D12" s="10"/>
@@ -1356,7 +1353,7 @@
     </x:row>
     <x:row r="13" ht="15" customHeight="1">
       <x:c r="A13" s="13" t="s">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B13" s="12" t="str">
         <x:v>本表为最终合并结果；如需修改，请保留本版本并另建新版本。</x:v>
@@ -1370,7 +1367,7 @@
     </x:row>
     <x:row r="14" ht="15" customHeight="1">
       <x:c r="A14" s="13" t="s">
-        <x:v>15</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B14" s="12" t="str">
         <x:v>双方原始标签、正式 project_label、adjudicated_label 和裁决理由均已保留。</x:v>
@@ -1384,10 +1381,10 @@
     </x:row>
     <x:row r="15" ht="15" customHeight="1">
       <x:c r="A15" s="13" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B15" s="12" t="s">
         <x:v>16</x:v>
-      </x:c>
-      <x:c r="B15" s="12" t="s">
-        <x:v>17</x:v>
       </x:c>
       <x:c r="C15" s="10"/>
       <x:c r="D15" s="10"/>
@@ -1716,7 +1713,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI5" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ5" s="7" t="str">
         <x:f t="shared" ref="AJ5:AJ24" si="0">IF(COUNTA(W5:AF5)=10,"已双标","待填写")</x:f>
@@ -1827,7 +1824,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI6" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ6" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -1938,7 +1935,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI7" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ7" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2049,7 +2046,7 @@
         <x:v>IRRELEVANT</x:v>
       </x:c>
       <x:c r="AI8" s="6" t="str">
-        <x:v>双方一致（IRRELEVANT）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（IRRELEVANT）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ8" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2160,7 +2157,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI9" s="6" t="str">
-        <x:v>陈明进标 ACCURATE，李云标 NOT_ACCURATE。被引摘要只说明化生性乳腺癌具有化疗耐药性，没有直接比较其标准化疗反应与传统TNBC，暂裁为 NOT_ACCURATE；证据状态仍为待定位。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>陈明进标 ACCURATE，李云标 NOT_ACCURATE。被引摘要只说明化生性乳腺癌具有化疗耐药性，没有直接比较其标准化疗反应与传统TNBC，最终裁决为 NOT_ACCURATE；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ9" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2271,7 +2268,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI10" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ10" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2382,7 +2379,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI11" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ11" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2493,7 +2490,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI12" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ12" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2604,7 +2601,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI13" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ13" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2715,7 +2712,7 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="AI14" s="6" t="str">
-        <x:v>双方一致（ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ14" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2826,7 +2823,7 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="AI15" s="6" t="str">
-        <x:v>双方一致（ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ15" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -2937,7 +2934,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI16" s="6" t="str">
-        <x:v>陈明进标 ACCURATE，李云标 NOT_ACCURATE。被引摘要只显示脂肪含量是单项研究的属性之一，不能支持‘已被多位研究者广泛研究’，暂裁为 NOT_ACCURATE；证据状态仍为待定位。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>陈明进标 ACCURATE，李云标 NOT_ACCURATE。被引摘要只显示脂肪含量是单项研究的属性之一，不能支持‘已被多位研究者广泛研究’，最终裁决为 NOT_ACCURATE；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ16" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3048,7 +3045,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI17" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ17" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3159,7 +3156,7 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="AI18" s="6" t="str">
-        <x:v>双方一致（ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ18" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3270,7 +3267,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI19" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ19" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3381,7 +3378,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI20" s="6" t="str">
-        <x:v>双方一致（统一 NOT-ACCURATE 为 NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（统一 NOT-ACCURATE 为 NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ20" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3492,7 +3489,7 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="AI21" s="6" t="str">
-        <x:v>双方一致（ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ21" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3603,7 +3600,7 @@
         <x:v>ACCURATE</x:v>
       </x:c>
       <x:c r="AI22" s="6" t="str">
-        <x:v>双方一致（ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ22" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3714,7 +3711,7 @@
         <x:v>NOT_ACCURATE</x:v>
       </x:c>
       <x:c r="AI23" s="6" t="str">
-        <x:v>双方一致（NOT_ACCURATE）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（NOT_ACCURATE）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ23" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3825,7 +3822,7 @@
         <x:v>IRRELEVANT</x:v>
       </x:c>
       <x:c r="AI24" s="6" t="str">
-        <x:v>双方一致（IRRELEVANT）；证据状态仍为待定位，暂不写入正式 project_label。；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
+        <x:v>双方一致（IRRELEVANT）；证据定位已完成，且已确认与现有 train/dev/test、调参和评测集无重叠，写入最终 project_label。</x:v>
       </x:c>
       <x:c r="AJ24" s="7" t="str">
         <x:f t="shared" si="0"/>
@@ -3865,7 +3862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bb853bc15d3456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cdd751bd3374389"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
ly: add row-level delivery index and status tables
</commit_message>
<xml_diff>
--- a/results/ly/task3_natural_trial/pmc_oa_v2_final_trial_set_v3_2026-10-04.xlsx
+++ b/results/ly/task3_natural_trial/pmc_oa_v2_final_trial_set_v3_2026-10-04.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Rd2a9a5c0088f4b65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Re0da84f8729c48f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Protocol" sheetId="1" r:id="Ra317f4da0a774568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blind_Annotation" sheetId="2" r:id="Ra7ee31dc03f24fdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1491,12 +1491,12 @@
   <x:sheetData>
     <x:row r="1" ht="18">
       <x:c r="A1" s="1" t="str">
-        <x:v>PMC natural 候选标注合并与暂定裁决（20 条）</x:v>
+        <x:v>PMC natural 候选标注合并与最终试标集 v3（20 条）</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2" t="str">
-        <x:v>已合并双方原值；adjudicated_label 为证据定位完成前的暂定语义裁决，project_label 暂留空。</x:v>
+        <x:v>已合并双方原始值；20 条证据均已定位，已完成最终裁决和数据集去重确认；project_label 已写入。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
@@ -1717,7 +1717,7 @@
       </x:c>
       <x:c r="AJ5" s="7" t="str">
         <x:f t="shared" ref="AJ5:AJ24" si="0">IF(COUNTA(W5:AF5)=10,"已双标","待填写")</x:f>
-        <x:v>已完成双人标注、证据定位、最终裁决与去重确认</x:v>
+        <x:v>已双标</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="409.5" customHeight="1">
@@ -3862,7 +3862,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3cdd751bd3374389"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc3bd8fa68dc4ef7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>